<commit_message>
1.update the readme, add pcb config info 2.update the bom.
</commit_message>
<xml_diff>
--- a/v1/bom_zh.xlsx
+++ b/v1/bom_zh.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\develop\my_workspace\self_playing_ruler\v1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DEV\project\self_playing_ruler\v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6953B557-13A2-49C9-8C72-DC65E1A93D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798D3140-F84A-45F1-B281-43D326624F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="77">
   <si>
     <t>类别</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -289,10 +292,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>贴片N-MOSS管（参考型号a03400a）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>润滑脂</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -321,6 +320,22 @@
   </si>
   <si>
     <t>drv8825/a4988步进电机驱动模块</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>贴片电容1uF</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>贴片电阻10K</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>贴片电阻150K</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>负载开关SGM2521YS8G/TR</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -732,7 +747,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.6640625" style="10"/>
@@ -805,7 +820,7 @@
         <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -829,7 +844,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -1117,7 +1132,7 @@
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -1366,7 +1381,7 @@
         <v>63</v>
       </c>
       <c r="C26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D26" t="s">
         <v>60</v>
@@ -1393,7 +1408,7 @@
         <v>63</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D27" t="s">
         <v>25</v>
@@ -1409,7 +1424,7 @@
         <v>0.60000000000000009</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -1420,7 +1435,7 @@
         <v>63</v>
       </c>
       <c r="C28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -1433,7 +1448,7 @@
         <v>0.06</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
@@ -1510,27 +1525,90 @@
         <v>63</v>
       </c>
       <c r="C32" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32">
-        <v>0.15</v>
+        <v>5</v>
       </c>
       <c r="G32">
-        <f>E32*F32</f>
-        <v>0.15</v>
+        <f t="shared" ref="G32:G35" si="1">E32*F32</f>
+        <v>5</v>
       </c>
       <c r="H32" s="9"/>
     </row>
-    <row r="34" spans="6:7" x14ac:dyDescent="0.3">
-      <c r="F34" t="s">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" t="s">
+        <v>73</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <v>0.05</v>
+      </c>
+      <c r="G33">
+        <f>E33*F33</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" t="s">
+        <v>74</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
+        <v>0.05</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" t="s">
+        <v>75</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
+        <v>0.05</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F37" t="s">
         <v>59</v>
       </c>
-      <c r="G34">
-        <f>SUM(G2:G33)</f>
-        <v>94.14</v>
+      <c r="G37">
+        <f>SUM(G2:G29)</f>
+        <v>93.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>